<commit_message>
Add property-price term to NPL and revise Adverse 1 property path
- dofile_fixed.do: judgmental property effect on NPL (global e_prop = -0.429,
  Prospera's summed elasticity, evenly over lags 1-4), added as a static term
  on top of the dynamic NPL core; e_prop reported in the Assumptions sheet.
- Solvency ST.xlsx, Scenario 2: d_property set to the midpoint between
  Baseline and Adverse 2 (F2:F7, values).
- CHANGELOG/README: rationale, before/after results, k_stress notes.
- Re-run outputs for v3 (intermediate/fixed, output/fixed) and the
  alternative logit model.

Adverse 2 NPL spread vs baseline 0.27 -> 0.75 pp; CAR end 22.47/21.88/21.11;
banks with CAR < 8% unchanged (Adverse 2: BINA, BCIC).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/Solvency ST.xlsx
+++ b/input/Solvency ST.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="533" documentId="13_ncr:1_{730491FC-1CE6-492F-A50E-63A683B2DED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D076EE6E-345D-4A14-8DEA-83468ED8B597}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Haircut" sheetId="7" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="Presentation" sheetId="8" r:id="rId6"/>
     <sheet name="Parameters" sheetId="9" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="135" uniqueCount="57">
   <si>
     <t>Dates</t>
   </si>
@@ -218,11 +218,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,000%"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -279,17 +279,17 @@
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4586,7 +4586,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
@@ -4604,7 +4604,7 @@
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+            <a:ext xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8BE0E6CE-BEDC-1810-2B96-D0B1E422AFBE}"/>
             </a:ext>
           </a:extLst>
@@ -4640,7 +4640,7 @@
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+            <a:ext xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E8DFBD17-C3E0-E7FF-2570-A92D2E1AC667}"/>
             </a:ext>
           </a:extLst>
@@ -4676,7 +4676,7 @@
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="5" name="Chart 4">
           <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+            <a:ext xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA0F8DD8-8908-137A-C04B-E836460606C2}"/>
             </a:ext>
           </a:extLst>
@@ -4712,7 +4712,7 @@
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="6" name="Chart 5">
           <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+            <a:ext xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{628EF41E-C1C4-0965-B4BA-6157B09ECC61}"/>
             </a:ext>
           </a:extLst>
@@ -4735,7 +4735,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -4886,7 +4886,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -4910,9 +4910,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -4936,7 +4936,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -4971,7 +4971,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -4989,7 +4989,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -5014,7 +5014,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -5072,14 +5072,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6488248C-5E8B-4193-A522-ACE31EF6A39B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6488248C-5E8B-4193-A522-ACE31EF6A39B}">
   <dimension ref="A1:J22"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.265625" customWidth="1"/>
+    <col min="1" max="1" width="11.265625" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -5102,7 +5102,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -5119,7 +5119,7 @@
         <v>0.1251447</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.45">
       <c r="E3" t="s">
         <v>29</v>
       </c>
@@ -5127,7 +5127,7 @@
         <v>8.4910200000000005E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.45">
       <c r="A4" s="11" t="s">
         <v>10</v>
       </c>
@@ -5138,7 +5138,7 @@
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -5170,7 +5170,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>46203</v>
       </c>
@@ -5210,7 +5210,7 @@
         <v>0.28680014790425773</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <v>46295</v>
       </c>
@@ -5250,7 +5250,7 @@
         <v>0.28680014790425773</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>46387</v>
       </c>
@@ -5290,7 +5290,7 @@
         <v>0.28680014790425773</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>46477</v>
       </c>
@@ -5330,7 +5330,7 @@
         <v>0.28680014790425773</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.45">
       <c r="A10" s="3">
         <v>46568</v>
       </c>
@@ -5370,7 +5370,7 @@
         <v>0.28680014790425773</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.45">
       <c r="A11" s="3">
         <v>46660</v>
       </c>
@@ -5410,7 +5410,7 @@
         <v>0.28680014790425773</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.45">
       <c r="A12" s="3">
         <v>46752</v>
       </c>
@@ -5450,11 +5450,11 @@
         <v>0.28680014790425773</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.45">
       <c r="A13" s="1"/>
       <c r="B13" s="7"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
         <v>12</v>
       </c>
@@ -5465,7 +5465,7 @@
       <c r="F14" s="11"/>
       <c r="G14" s="11"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -5497,7 +5497,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
         <v>46203</v>
       </c>
@@ -5537,7 +5537,7 @@
         <v>0.57360029580851546</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <v>46295</v>
       </c>
@@ -5577,7 +5577,7 @@
         <v>0.57360029580851546</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
         <v>46387</v>
       </c>
@@ -5617,7 +5617,7 @@
         <v>0.57360029580851546</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
         <v>46477</v>
       </c>
@@ -5657,7 +5657,7 @@
         <v>0.57360029580851546</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.45">
       <c r="A20" s="3">
         <v>46568</v>
       </c>
@@ -5697,7 +5697,7 @@
         <v>0.57360029580851546</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.45">
       <c r="A21" s="3">
         <v>46660</v>
       </c>
@@ -5737,7 +5737,7 @@
         <v>0.57360029580851546</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.45">
       <c r="A22" s="3">
         <v>46752</v>
       </c>
@@ -5787,14 +5787,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E011A9C0-5B3E-4E01-ADE7-D48E04462C58}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E011A9C0-5B3E-4E01-ADE7-D48E04462C58}">
   <dimension ref="A1:L50"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.19921875" customWidth="1"/>
+    <col min="1" max="1" width="11.19921875" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5832,7 +5832,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.45">
       <c r="A2" s="3">
         <v>41820</v>
       </c>
@@ -5863,7 +5863,7 @@
         <v>8.2129999999999992</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.45">
       <c r="A3" s="3">
         <v>41912</v>
       </c>
@@ -5905,7 +5905,7 @@
         <v>8.5210000000000008</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.45">
       <c r="A4" s="3">
         <v>42004</v>
       </c>
@@ -5947,7 +5947,7 @@
         <v>7.7960000000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.45">
       <c r="A5" s="3">
         <v>42094</v>
       </c>
@@ -5989,7 +5989,7 @@
         <v>7.5570000000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.45">
       <c r="A6" s="3">
         <v>42185</v>
       </c>
@@ -6031,7 +6031,7 @@
         <v>8.3829999999999991</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.45">
       <c r="A7" s="3">
         <v>42277</v>
       </c>
@@ -6073,7 +6073,7 @@
         <v>9.6910000000000007</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.45">
       <c r="A8" s="3">
         <v>42369</v>
       </c>
@@ -6115,7 +6115,7 @@
         <v>8.9930000000000003</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.45">
       <c r="A9" s="3">
         <v>42460</v>
       </c>
@@ -6157,7 +6157,7 @@
         <v>7.6680000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.45">
       <c r="A10" s="3">
         <v>42551</v>
       </c>
@@ -6199,7 +6199,7 @@
         <v>7.4530000000000003</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.45">
       <c r="A11" s="3">
         <v>42643</v>
       </c>
@@ -6241,7 +6241,7 @@
         <v>7.0609999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.45">
       <c r="A12" s="3">
         <v>42735</v>
       </c>
@@ -6283,7 +6283,7 @@
         <v>7.9729999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.45">
       <c r="A13" s="3">
         <v>42825</v>
       </c>
@@ -6325,7 +6325,7 @@
         <v>7.0430000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.45">
       <c r="A14" s="3">
         <v>42916</v>
       </c>
@@ -6367,7 +6367,7 @@
         <v>6.8289999999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.45">
       <c r="A15" s="3">
         <v>43008</v>
       </c>
@@ -6409,7 +6409,7 @@
         <v>6.4969999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.45">
       <c r="A16" s="3">
         <v>43100</v>
       </c>
@@ -6451,7 +6451,7 @@
         <v>6.319</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.45">
       <c r="A17" s="3">
         <v>43190</v>
       </c>
@@ -6493,7 +6493,7 @@
         <v>6.6749999999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.45">
       <c r="A18" s="3">
         <v>43281</v>
       </c>
@@ -6535,7 +6535,7 @@
         <v>7.7969999999999997</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.45">
       <c r="A19" s="3">
         <v>43373</v>
       </c>
@@ -6577,7 +6577,7 @@
         <v>8.1150000000000002</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.45">
       <c r="A20" s="3">
         <v>43465</v>
       </c>
@@ -6619,7 +6619,7 @@
         <v>8.0250000000000004</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.45">
       <c r="A21" s="3">
         <v>43555</v>
       </c>
@@ -6661,7 +6661,7 @@
         <v>7.633</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.45">
       <c r="A22" s="3">
         <v>43646</v>
       </c>
@@ -6703,7 +6703,7 @@
         <v>7.3680000000000003</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.45">
       <c r="A23" s="3">
         <v>43738</v>
       </c>
@@ -6745,7 +6745,7 @@
         <v>7.2880000000000003</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.45">
       <c r="A24" s="3">
         <v>43830</v>
       </c>
@@ -6787,7 +6787,7 @@
         <v>7.0629999999999997</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.45">
       <c r="A25" s="3">
         <v>43921</v>
       </c>
@@ -6829,7 +6829,7 @@
         <v>7.9139999999999997</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.45">
       <c r="A26" s="3">
         <v>44012</v>
       </c>
@@ -6871,7 +6871,7 @@
         <v>7.2089999999999996</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.45">
       <c r="A27" s="3">
         <v>44104</v>
       </c>
@@ -6913,7 +6913,7 @@
         <v>6.9619999999999997</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.45">
       <c r="A28" s="3">
         <v>44196</v>
       </c>
@@ -6955,7 +6955,7 @@
         <v>5.8860000000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.45">
       <c r="A29" s="3">
         <v>44286</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>6.7770000000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.45">
       <c r="A30" s="3">
         <v>44377</v>
       </c>
@@ -7039,7 +7039,7 @@
         <v>6.59</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.45">
       <c r="A31" s="3">
         <v>44469</v>
       </c>
@@ -7081,7 +7081,7 @@
         <v>6.2610000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.45">
       <c r="A32" s="3">
         <v>44561</v>
       </c>
@@ -7123,7 +7123,7 @@
         <v>6.3819999999999997</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.45">
       <c r="A33" s="3">
         <v>44651</v>
       </c>
@@ -7164,7 +7164,7 @@
         <v>6.7380000000000004</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.45">
       <c r="A34" s="3">
         <v>44742</v>
       </c>
@@ -7205,7 +7205,7 @@
         <v>7.22</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.45">
       <c r="A35" s="3">
         <v>44834</v>
       </c>
@@ -7246,7 +7246,7 @@
         <v>7.3730000000000002</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.45">
       <c r="A36" s="3">
         <v>44926</v>
       </c>
@@ -7287,7 +7287,7 @@
         <v>6.94</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.45">
       <c r="A37" s="3">
         <v>45016</v>
       </c>
@@ -7328,7 +7328,7 @@
         <v>6.7930000000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.45">
       <c r="A38" s="3">
         <v>45107</v>
       </c>
@@ -7368,7 +7368,7 @@
         <v>6.2610000000000001</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.45">
       <c r="A39" s="3">
         <v>45199</v>
       </c>
@@ -7408,7 +7408,7 @@
         <v>6.9139999999999997</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.45">
       <c r="A40" s="3">
         <v>45291</v>
       </c>
@@ -7448,7 +7448,7 @@
         <v>6.48</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.45">
       <c r="A41" s="3">
         <v>45382</v>
       </c>
@@ -7488,7 +7488,7 @@
         <v>6.6929999999999996</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.45">
       <c r="A42" s="1">
         <v>45473</v>
       </c>
@@ -7528,7 +7528,7 @@
         <v>7.0730000000000004</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.45">
       <c r="A43" s="1">
         <v>45565</v>
       </c>
@@ -7567,7 +7567,7 @@
         <v>6.4530000000000003</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.45">
       <c r="A44" s="1">
         <v>45657</v>
       </c>
@@ -7606,7 +7606,7 @@
         <v>6.9969999999999999</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.45">
       <c r="A45" s="1">
         <v>45747</v>
       </c>
@@ -7645,7 +7645,7 @@
         <v>7.0039999999999996</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.45">
       <c r="A46" s="1">
         <v>45838</v>
       </c>
@@ -7684,7 +7684,7 @@
         <v>6.6280000000000001</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.45">
       <c r="A47" s="1">
         <v>45930</v>
       </c>
@@ -7723,7 +7723,7 @@
         <v>6.367</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.45">
       <c r="A48" s="1">
         <v>46022</v>
       </c>
@@ -7762,7 +7762,7 @@
         <v>6.07</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.45">
       <c r="A49" s="1">
         <v>46112</v>
       </c>
@@ -7801,7 +7801,7 @@
         <v>6.8550000000000004</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.45">
       <c r="A50" s="1">
         <v>46203</v>
       </c>
@@ -7846,14 +7846,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32FA261B-C9CE-4B99-BBE1-3127CE69A6D8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32FA261B-C9CE-4B99-BBE1-3127CE69A6D8}">
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.06640625" customWidth="1"/>
+    <col min="1" max="1" width="11.06640625" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7888,7 +7888,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.45">
       <c r="A2" s="3">
         <v>46295</v>
       </c>
@@ -7925,7 +7925,7 @@
         <v>7.0949999999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.45">
       <c r="A3" s="3">
         <v>46387</v>
       </c>
@@ -7964,7 +7964,7 @@
         <v>7.0583484006411981</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.45">
       <c r="A4" s="3">
         <v>46477</v>
       </c>
@@ -8003,7 +8003,7 @@
         <v>6.9311174759889447</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.45">
       <c r="A5" s="3">
         <v>46568</v>
       </c>
@@ -8042,7 +8042,7 @@
         <v>6.8514492897441333</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.45">
       <c r="A6" s="3">
         <v>46660</v>
       </c>
@@ -8081,7 +8081,7 @@
         <v>6.8027900161766475</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.45">
       <c r="A7" s="3">
         <v>46752</v>
       </c>
@@ -8127,14 +8127,14 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{922E0524-F95C-44FA-8CCF-CDBA108E8470}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{922E0524-F95C-44FA-8CCF-CDBA108E8470}">
   <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.06640625" customWidth="1"/>
+    <col min="1" max="1" width="12.06640625" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8166,7 +8166,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.45">
       <c r="A2" s="3">
         <v>46295</v>
       </c>
@@ -8187,8 +8187,7 @@
         <v>18207.497266083861</v>
       </c>
       <c r="F2">
-        <f>Macro!J50-Haircut!I7</f>
-        <v>0.20186731553845472</v>
+        <v>0.18186731553845159</v>
       </c>
       <c r="G2">
         <f>-Haircut!$H$1*(J2-Macro!L50)</f>
@@ -8206,7 +8205,7 @@
         <v>7.3747358193391319</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.45">
       <c r="A3" s="3">
         <v>46387</v>
       </c>
@@ -8227,7 +8226,7 @@
         <v>18537.994532167722</v>
       </c>
       <c r="F3">
-        <v>0.35999999999998522</v>
+        <v>-0.57000000000000739</v>
       </c>
       <c r="G3">
         <f>-Haircut!$H$1*(J3-J2)</f>
@@ -8245,7 +8244,7 @@
         <v>7.6218899653449848</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.45">
       <c r="A4" s="3">
         <v>46477</v>
       </c>
@@ -8266,7 +8265,7 @@
         <v>18868.491798251584</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>-1.2000000000000029</v>
       </c>
       <c r="G4">
         <f>-Haircut!$H$1*(J4-J3)</f>
@@ -8284,7 +8283,7 @@
         <v>7.8663448860599745</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.45">
       <c r="A5" s="3">
         <v>46568</v>
       </c>
@@ -8305,7 +8304,7 @@
         <v>19198.989064335445</v>
       </c>
       <c r="F5">
-        <v>0.1071561619203264</v>
+        <v>-1.1599999999999966</v>
       </c>
       <c r="G5">
         <f>-Haircut!$H$1*(J5-J4)</f>
@@ -8323,7 +8322,7 @@
         <v>8.1081943260668989</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.45">
       <c r="A6" s="3">
         <v>46660</v>
       </c>
@@ -8344,7 +8343,7 @@
         <v>19529.486330419306</v>
       </c>
       <c r="F6">
-        <v>-0.22045845077289927</v>
+        <v>-0.43500000000000227</v>
       </c>
       <c r="G6">
         <f>-Haircut!$H$1*(J6-J5)</f>
@@ -8362,7 +8361,7 @@
         <v>8.3475272295400522</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.45">
       <c r="A7" s="3">
         <v>46752</v>
       </c>
@@ -8383,7 +8382,7 @@
         <v>19859.983596503167</v>
       </c>
       <c r="F7">
-        <v>-0.54807306346612494</v>
+        <v>-0.18499999999998806</v>
       </c>
       <c r="G7">
         <f>-Haircut!$H$1*(J7-J6)</f>
@@ -8407,14 +8406,14 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0364041A-325D-43C8-A7A5-E082D9FDD9D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0364041A-325D-43C8-A7A5-E082D9FDD9D5}">
   <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8446,7 +8445,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.45">
       <c r="A2" s="3">
         <v>46295</v>
       </c>
@@ -8486,7 +8485,7 @@
         <v>7.6516735166137781</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.45">
       <c r="A3" s="3">
         <v>46387</v>
       </c>
@@ -8525,7 +8524,7 @@
         <v>8.2273285311420761</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.45">
       <c r="A4" s="3">
         <v>46477</v>
       </c>
@@ -8564,7 +8563,7 @@
         <v>8.7929129213884618</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.45">
       <c r="A5" s="3">
         <v>46568</v>
       </c>
@@ -8603,7 +8602,7 @@
         <v>9.3490862529687853</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.45">
       <c r="A6" s="3">
         <v>46660</v>
       </c>
@@ -8642,7 +8641,7 @@
         <v>9.8964453444506724</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.45">
       <c r="A7" s="3">
         <v>46752</v>
       </c>
@@ -8687,11 +8686,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9AB7026-AA14-4A3C-BA72-E499094D6A1D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9AB7026-AA14-4A3C-BA72-E499094D6A1D}">
   <dimension ref="A1:D34"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -8705,7 +8704,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -8722,7 +8721,7 @@
         <v>5.29</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
@@ -8739,7 +8738,7 @@
         <v>4.1332363293974659</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>22</v>
       </c>
@@ -8756,7 +8755,7 @@
         <v>2.9764726587949313</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>23</v>
       </c>
@@ -8773,7 +8772,7 @@
         <v>1.8197089881923967</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -8790,7 +8789,7 @@
         <v>0.66294531758986208</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -8804,7 +8803,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>21</v>
       </c>
@@ -8821,7 +8820,7 @@
         <v>5.75</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
@@ -8838,7 +8837,7 @@
         <v>5.9879929095582476</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
@@ -8855,7 +8854,7 @@
         <v>6.2259858191164952</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
@@ -8872,7 +8871,7 @@
         <v>6.4639787286747428</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -8886,7 +8885,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -8901,7 +8900,7 @@
         <v>0.38586167999999077</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>21</v>
       </c>
@@ -8918,7 +8917,7 @@
         <v>0.11373463107690321</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>22</v>
       </c>
@@ -8935,7 +8934,7 @@
         <v>-1.3900000000000148</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>23</v>
       </c>
@@ -8952,7 +8951,7 @@
         <v>-2.6500000000000057</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>24</v>
       </c>
@@ -8969,7 +8968,7 @@
         <v>-2.5699999999999932</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>19</v>
       </c>
@@ -8983,7 +8982,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -9000,7 +8999,7 @@
         <v>-2.4683675830688889</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -9017,7 +9016,7 @@
         <v>-2.8782750726414896</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -9034,7 +9033,7 @@
         <v>-2.8279219512319287</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -9051,34 +9050,34 @@
         <v>-2.7808666579016172</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.45">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.45">
       <c r="A30" s="1"/>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.45">
       <c r="A31" s="1"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.45">
       <c r="A32" s="1"/>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.45">
       <c r="A33" s="1"/>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.45">
       <c r="A34" s="1"/>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -9091,15 +9090,15 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3CECDCA-61C7-4498-B1B8-1D2ECBC8866D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3CECDCA-61C7-4498-B1B8-1D2ECBC8866D}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="12.59765625" customWidth="1"/>
-    <col min="3" max="4" width="70.59765625" customWidth="1"/>
+    <col min="1" max="2" width="12.59765625" customWidth="true"/>
+    <col min="3" max="4" width="70.59765625" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>31</v>
       </c>
@@ -9113,7 +9112,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>35</v>
       </c>
@@ -9127,7 +9126,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -9141,7 +9140,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -9155,7 +9154,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -9170,7 +9169,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -9184,7 +9183,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>50</v>
       </c>
@@ -9198,7 +9197,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>52</v>
       </c>
@@ -9212,7 +9211,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>55</v>
       </c>

</xml_diff>

<commit_message>
Make Adverse 1 coherent and strengthen BI response in Adverse 2
- Solvency ST.xlsx, Scenario 2 (Adverse 1): BI rate +50 bp (was cut by 71 bp
  while the rupiah weakened and CPI rose above target); property at 50% of the
  Adverse 2 deviation from baseline.
- Scenario 3 (Adverse 2): BI rate +150 bp; property path reshaped so it does
  not recover while GDP is still falling (4Q total about -6.5%).
- SBN 10Y shifted by beta_rate x change in BI rate; d_price = -5 x dSBN 10Y.
  Columns C, F, G, J (rows 2-7) are now values.
- CHANGELOG updated; v3 outputs re-run.

End 2027Q2: NPL 2.26/2.67/3.08, CAR 22.47/21.80/21.03; banks with CAR < 8%
unchanged (Adverse 2: BINA, BCIC).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/Solvency ST.xlsx
+++ b/input/Solvency ST.xlsx
@@ -8175,7 +8175,6 @@
         <v>4.7116181646987325</v>
       </c>
       <c r="C2">
-        <f>'Scenario 1'!C2</f>
         <v>5.75</v>
       </c>
       <c r="D2">
@@ -8187,10 +8186,9 @@
         <v>18207.497266083861</v>
       </c>
       <c r="F2">
-        <v>0.18186731553845159</v>
+        <v>-0.125</v>
       </c>
       <c r="G2">
-        <f>-Haircut!$H$1*(J2-Macro!L50)</f>
         <v>-1.0836790966956578</v>
       </c>
       <c r="H2">
@@ -8201,7 +8199,6 @@
         <v>5.2481001479042577</v>
       </c>
       <c r="J2">
-        <f>'Scenario 1'!K2+Haircut!$F$1*(I2-'Scenario 1'!J2)+Haircut!$F$2*(C2-'Scenario 1'!C2)+Haircut!$F$3*100*LN(E2/'Scenario 1'!E2)</f>
         <v>7.3747358193391319</v>
       </c>
     </row>
@@ -8214,8 +8211,7 @@
         <v>4.133236329397465</v>
       </c>
       <c r="C3">
-        <f>C2-Haircut!D7</f>
-        <v>5.5120070904417524</v>
+        <v>6</v>
       </c>
       <c r="D3">
         <f>D2+Haircut!E7</f>
@@ -8226,11 +8222,10 @@
         <v>18537.994532167722</v>
       </c>
       <c r="F3">
-        <v>-0.57000000000000739</v>
+        <v>-0.625</v>
       </c>
       <c r="G3">
-        <f>-Haircut!$H$1*(J3-J2)</f>
-        <v>-1.2357707300292642</v>
+        <v>-1.5411193613732355</v>
       </c>
       <c r="H3">
         <v>267</v>
@@ -8240,8 +8235,7 @@
         <v>5.5349002958085158</v>
       </c>
       <c r="J3">
-        <f>J2+Haircut!$F$1*(I3-I2)+Haircut!$F$2*(C3-C2)+Haircut!$F$3*100*LN(E3/E2)</f>
-        <v>7.6218899653449848</v>
+        <v>7.682959691613779</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.45">
@@ -8253,8 +8247,7 @@
         <v>3.5548544940961975</v>
       </c>
       <c r="C4">
-        <f>C3-Haircut!D8</f>
-        <v>5.2740141808835048</v>
+        <v>6.25</v>
       </c>
       <c r="D4">
         <f>D3+Haircut!E8</f>
@@ -8265,11 +8258,10 @@
         <v>18868.491798251584</v>
       </c>
       <c r="F4">
-        <v>-1.2000000000000029</v>
+        <v>-0.875</v>
       </c>
       <c r="G4">
-        <f>-Haircut!$H$1*(J4-J3)</f>
-        <v>-1.2222746035749488</v>
+        <v>-1.5276232349189156</v>
       </c>
       <c r="H4">
         <v>268</v>
@@ -8279,8 +8271,7 @@
         <v>5.821700443712774</v>
       </c>
       <c r="J4">
-        <f>J3+Haircut!$F$1*(I4-I3)+Haircut!$F$2*(C4-C3)+Haircut!$F$3*100*LN(E4/E3)</f>
-        <v>7.8663448860599745</v>
+        <v>7.9884843385975621</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.45">
@@ -8292,8 +8283,7 @@
         <v>2.9764726587949299</v>
       </c>
       <c r="C5">
-        <f>C4-Haircut!D9</f>
-        <v>5.0360212713252572</v>
+        <v>6.25</v>
       </c>
       <c r="D5">
         <f>D4+Haircut!E9</f>
@@ -8304,11 +8294,10 @@
         <v>19198.989064335445</v>
       </c>
       <c r="F5">
-        <v>-1.1599999999999966</v>
+        <v>-1.125</v>
       </c>
       <c r="G5">
-        <f>-Haircut!$H$1*(J5-J4)</f>
-        <v>-1.2092472000346222</v>
+        <v>-1.358164956378598</v>
       </c>
       <c r="H5">
         <v>269</v>
@@ -8318,8 +8307,7 @@
         <v>6.1085005916170321</v>
       </c>
       <c r="J5">
-        <f>J4+Haircut!$F$1*(I5-I4)+Haircut!$F$2*(C5-C4)+Haircut!$F$3*100*LN(E5/E4)</f>
-        <v>8.1081943260668989</v>
+        <v>8.2601173298732817</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.45">
@@ -8331,8 +8319,7 @@
         <v>2.3980908234936624</v>
       </c>
       <c r="C6">
-        <f>C5-Haircut!D10</f>
-        <v>4.7980283617670096</v>
+        <v>6.25</v>
       </c>
       <c r="D6">
         <f>'Scenario 2'!D5+Haircut!E10</f>
@@ -8343,11 +8330,10 @@
         <v>19529.486330419306</v>
       </c>
       <c r="F6">
-        <v>-0.43500000000000227</v>
+        <v>-1.125</v>
       </c>
       <c r="G6">
-        <f>-Haircut!$H$1*(J6-J5)</f>
-        <v>-1.1966645173657664</v>
+        <v>-1.3455822737097289</v>
       </c>
       <c r="H6">
         <v>270</v>
@@ -8357,8 +8343,7 @@
         <v>6.3953007395212902</v>
       </c>
       <c r="J6">
-        <f>J5+Haircut!$F$1*(I6-I5)+Haircut!$F$2*(C6-C5)+Haircut!$F$3*100*LN(E6/E5)</f>
-        <v>8.3475272295400522</v>
+        <v>8.5292337846152275</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.45">
@@ -8370,8 +8355,7 @@
         <v>1.8197089881923951</v>
       </c>
       <c r="C7">
-        <f>C6-Haircut!D11</f>
-        <v>4.5600354522087621</v>
+        <v>6.25</v>
       </c>
       <c r="D7">
         <f>D6+Haircut!E11</f>
@@ -8382,11 +8366,10 @@
         <v>19859.983596503167</v>
       </c>
       <c r="F7">
-        <v>-0.18499999999998806</v>
+        <v>-0.875</v>
       </c>
       <c r="G7">
-        <f>-Haircut!$H$1*(J7-J6)</f>
-        <v>-1.1845041648342658</v>
+        <v>-1.3334219211782372</v>
       </c>
       <c r="H7">
         <v>271</v>
@@ -8396,8 +8379,7 @@
         <v>6.6821008874255483</v>
       </c>
       <c r="J7">
-        <f>J6+Haircut!$F$1*(I7-I6)+Haircut!$F$2*(C7-C6)+Haircut!$F$3*100*LN(E7/E6)</f>
-        <v>8.5844280625069054</v>
+        <v>8.795918168850875</v>
       </c>
     </row>
   </sheetData>
@@ -8454,8 +8436,7 @@
         <v>4.1332363293974659</v>
       </c>
       <c r="C2">
-        <f>'Scenario 1'!C2</f>
-        <v>5.75</v>
+        <v>6</v>
       </c>
       <c r="D2">
         <f>Macro!D50+Haircut!E17</f>
@@ -8466,12 +8447,10 @@
         <v>18537.994532167722</v>
       </c>
       <c r="F2">
-        <f>Macro!J50-Haircut!I17</f>
-        <v>0.11373463107690321</v>
+        <v>-0.5</v>
       </c>
       <c r="G2">
-        <f>-Haircut!$H$1*(J2-Macro!L50)</f>
-        <v>-2.4683675830688889</v>
+        <v>-2.6247984580688888</v>
       </c>
       <c r="H2">
         <v>266</v>
@@ -8481,8 +8460,7 @@
         <v>5.5349002958085149</v>
       </c>
       <c r="J2">
-        <f>'Scenario 1'!K2+Haircut!$F$1*(I2-'Scenario 1'!J2)+Haircut!$F$2*(C2-'Scenario 1'!C2)+Haircut!$F$3*100*LN(E2/'Scenario 1'!E2)</f>
-        <v>7.6516735166137781</v>
+        <v>7.6829596916137781</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.45">
@@ -8494,8 +8472,7 @@
         <v>2.9764726587949313</v>
       </c>
       <c r="C3">
-        <f>C2+Haircut!D8</f>
-        <v>5.9879929095582476</v>
+        <v>6.5</v>
       </c>
       <c r="D3">
         <f>D2+Haircut!E17</f>
@@ -8506,11 +8483,10 @@
         <v>19198.989064335445</v>
       </c>
       <c r="F3">
-        <v>-1.3900000000000148</v>
+        <v>-1.5</v>
       </c>
       <c r="G3">
-        <f>-Haircut!$H$1*(J3-J2)</f>
-        <v>-2.8782750726414896</v>
+        <v>-3.0422190662975179</v>
       </c>
       <c r="H3">
         <v>267</v>
@@ -8520,8 +8496,7 @@
         <v>6.1085005916170303</v>
       </c>
       <c r="J3">
-        <f>J2+Haircut!$F$1*(I3-I2)+Haircut!$F$2*(C3-C2)+Haircut!$F$3*100*LN(E3/E2)</f>
-        <v>8.2273285311420761</v>
+        <v>8.2914035048732817</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.45">
@@ -8533,8 +8508,7 @@
         <v>1.8197089881923967</v>
       </c>
       <c r="C4">
-        <f>C3+Haircut!D9</f>
-        <v>6.2259858191164952</v>
+        <v>7</v>
       </c>
       <c r="D4">
         <f>D3+Haircut!E18</f>
@@ -8545,11 +8519,10 @@
         <v>19859.983596503167</v>
       </c>
       <c r="F4">
-        <v>-2.6500000000000057</v>
+        <v>-2</v>
       </c>
       <c r="G4">
-        <f>-Haircut!$H$1*(J4-J3)</f>
-        <v>-2.8279219512319287</v>
+        <v>-2.991865944887957</v>
       </c>
       <c r="H4">
         <v>268</v>
@@ -8559,8 +8532,7 @@
         <v>6.6821008874255456</v>
       </c>
       <c r="J4">
-        <f>J3+Haircut!$F$1*(I4-I3)+Haircut!$F$2*(C4-C3)+Haircut!$F$3*100*LN(E4/E3)</f>
-        <v>8.7929129213884618</v>
+        <v>8.8897766938508731</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.45">
@@ -8572,8 +8544,7 @@
         <v>0.66294531758986208</v>
       </c>
       <c r="C5">
-        <f>C4+Haircut!D10</f>
-        <v>6.4639787286747428</v>
+        <v>7.25</v>
       </c>
       <c r="D5">
         <f>D4+Haircut!E19</f>
@@ -8584,11 +8555,10 @@
         <v>20520.978128670889</v>
       </c>
       <c r="F5">
-        <v>-2.5699999999999932</v>
+        <v>-2.5</v>
       </c>
       <c r="G5">
-        <f>-Haircut!$H$1*(J5-J4)</f>
-        <v>-2.7808666579016172</v>
+        <v>-2.7883797765576546</v>
       </c>
       <c r="H5">
         <v>269</v>
@@ -8598,8 +8568,7 @@
         <v>7.255701183234061</v>
       </c>
       <c r="J5">
-        <f>J4+Haircut!$F$1*(I5-I4)+Haircut!$F$2*(C5-C4)+Haircut!$F$3*100*LN(E5/E4)</f>
-        <v>9.3490862529687853</v>
+        <v>9.447452649162404</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.45">
@@ -8611,8 +8580,7 @@
         <v>-0.49381835301267252</v>
       </c>
       <c r="C6">
-        <f>'Scenario 3'!C5+Haircut!D11</f>
-        <v>6.7019716382329904</v>
+        <v>7.25</v>
       </c>
       <c r="D6">
         <f>'Scenario 3'!D5+Haircut!E20</f>
@@ -8623,11 +8591,10 @@
         <v>21181.972660838612</v>
       </c>
       <c r="F6">
-        <v>-1.1200000000000045</v>
+        <v>-2.5</v>
       </c>
       <c r="G6">
-        <f>-Haircut!$H$1*(J6-J5)</f>
-        <v>-2.7367954574094355</v>
+        <v>-2.5878777010654641</v>
       </c>
       <c r="H6">
         <v>270</v>
@@ -8637,8 +8604,7 @@
         <v>7.8293014790425763</v>
       </c>
       <c r="J6">
-        <f>J5+Haircut!$F$1*(I6-I5)+Haircut!$F$2*(C6-C5)+Haircut!$F$3*100*LN(E6/E5)</f>
-        <v>9.8964453444506724</v>
+        <v>9.9650281893754968</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.45">
@@ -8650,8 +8616,7 @@
         <v>-1.6505820236152071</v>
       </c>
       <c r="C7">
-        <f>C6+Haircut!D12</f>
-        <v>6.9399645477912379</v>
+        <v>7.25</v>
       </c>
       <c r="D7">
         <f>D6+Haircut!E21</f>
@@ -8662,11 +8627,10 @@
         <v>21842.967193006334</v>
       </c>
       <c r="F7">
-        <v>-0.61999999999997613</v>
+        <v>-2</v>
       </c>
       <c r="G7">
-        <f>-Haircut!$H$1*(J7-J6)</f>
-        <v>-2.6954331901687656</v>
+        <v>-2.5465154338247942</v>
       </c>
       <c r="H7">
         <v>271</v>
@@ -8676,8 +8640,7 @@
         <v>8.4029017748510917</v>
       </c>
       <c r="J7">
-        <f>J6+Haircut!$F$1*(I7-I6)+Haircut!$F$2*(C7-C6)+Haircut!$F$3*100*LN(E7/E6)</f>
-        <v>10.435531982484425</v>
+        <v>10.474331276140456</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Partial rate pass-through, overlay k 0.03, deck update
- Pass-through: beta_l 0.145 (product transmission x BI loan mix, May 2026),
  beta_d 0.694 (1-month deposit transmission applied to all funding; upper bound).
  Was 1.0 for both. Read from sheet Parameters; listed in Assumptions.
- k_stress 0.05 -> 0.03, calibrated so Adverse 2 credit loss matches the 2021Q1
  provisioning peak (10.5% of capital); data estimate ~0.02.
- Rerun: CAR 22.53 / 21.87 / 21.14, NPL 2.25 / 2.66 / 3.06, failures 0 / 0 / 2.
- Deck: all numbers updated, new pass-through slide, provision slide restated
  (base credit cost as anchor; stress via NPL response + overlay).
- CHANGELOG and README updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/Solvency ST.xlsx
+++ b/input/Solvency ST.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="135" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="142" uniqueCount="64">
   <si>
     <t>Dates</t>
   </si>
@@ -213,6 +213,27 @@
   </si>
   <si>
     <t>Corporate income tax rate</t>
+  </si>
+  <si>
+    <t>calibrated: Adverse 2 credit loss ~ 2021Q1 peak of 4-quarter provisions in our data (10.5% of capital); data-based estimate ~0.02</t>
+  </si>
+  <si>
+    <t>beta_l</t>
+  </si>
+  <si>
+    <t>Pass-through of BI rate changes to loan rates (share of the change)</t>
+  </si>
+  <si>
+    <t>Transmission table, 3 BI hiking episodes (2018-19, 2022-24, 2026), weighted by BI loan mix May 2026: working capital 42.3%, investment 30.5%, consumption 27.2% (consumption excl. 2018)</t>
+  </si>
+  <si>
+    <t>beta_d</t>
+  </si>
+  <si>
+    <t>Pass-through of BI rate changes to funding cost (share of the change)</t>
+  </si>
+  <si>
+    <t>Transmission of 1-month time deposits, average of the same 3 episodes; applied to all funding (upper bound for funding pressure)</t>
   </si>
 </sst>
 </file>
@@ -9054,7 +9075,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3CECDCA-61C7-4498-B1B8-1D2ECBC8866D}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="12.59765625" customWidth="true"/>
@@ -9165,13 +9186,13 @@
         <v>52</v>
       </c>
       <c r="B8">
-        <v>0.05</v>
+        <v>0.029999999999999999</v>
       </c>
       <c r="C8" t="s">
         <v>53</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.45">
@@ -9186,6 +9207,34 @@
       </c>
       <c r="D9" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10">
+        <v>0.14499999999999999</v>
+      </c>
+      <c r="C10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11">
+        <v>0.69399999999999995</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>